<commit_message>
Fixed leave data transformation
</commit_message>
<xml_diff>
--- a/SSIS-Project/Timesheets/Teolan/Teolan_Govender_June_Week02.xlsx
+++ b/SSIS-Project/Timesheets/Teolan/Teolan_Govender_June_Week02.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://northerndata-my.sharepoint.com/personal/teolan_govender_sambeconsulting_com/Documents/Documents/Timesheets and Leave/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_TeolanGovender_2026\SSIS-Project\Timesheets\Teolan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1725" documentId="13_ncr:1_{18456319-F974-4A60-AFC5-4E049C41B553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7E4DC1ED-355C-4B1A-A9E7-D0605C0173E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4463279A-9A75-43FD-9107-279F85556406}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{1C8F8026-B005-4B08-94D3-371A77F74D8F}"/>
+    <workbookView xWindow="4245" yWindow="2325" windowWidth="21600" windowHeight="11295" activeTab="7" xr2:uid="{1C8F8026-B005-4B08-94D3-371A77F74D8F}"/>
   </bookViews>
   <sheets>
     <sheet name="Apr" sheetId="10" r:id="rId1"/>
@@ -11570,7 +11570,7 @@
         <v>2</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>106</v>
+        <v>212</v>
       </c>
       <c r="C5" s="37"/>
       <c r="H5" s="40"/>
@@ -17233,10 +17233,10 @@
         <v>81</v>
       </c>
       <c r="B11" s="117">
-        <v>46094</v>
+        <v>46155</v>
       </c>
       <c r="C11" s="117">
-        <v>46095</v>
+        <v>46156</v>
       </c>
       <c r="D11" s="87">
         <v>1</v>

</xml_diff>